<commit_message>
fix: adapt code and config for new Excel format
- Remove old fixed_address_param_config files (replaced by new format)
- Update profile.yaml injection paths to new file names
- Fix load_commands: remove is_polling column (no longer in Excel)
- Fix load_commands: use wb[wb.sheetnames[0]] instead of wb.active
- Fix load_telemetry_packages: skip frame format sheets, handle '-' values
- Fix load_injections: adapt for new column format (same as telemetry)
- Add _safe_int / _safe_float helper methods for robust parsing
- Update profile.yaml sheet names (常规包1参数表 -> 常规包1)
- Copy new Excel files to profile directory
</commit_message>
<xml_diff>
--- a/profiles/ppcu_rs422/telemetry/遥测配置表.xlsx
+++ b/profiles/ppcu_rs422/telemetry/遥测配置表.xlsx
@@ -5,25 +5,25 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codex Workspace\01_Projects\项目文档\通讯协议\excel版遥测大表\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codex Workspace\02_Projects\项目文档\excel版遥测大表\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E57D0B7-4A2D-4F43-97B9-5AD5F196CBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50183941-7CF1-43E8-A2B9-AC4D8C570976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="常规包1参数表" sheetId="1" r:id="rId1"/>
-    <sheet name="常规包2参数表" sheetId="2" r:id="rId2"/>
-    <sheet name="查询包1参数表" sheetId="3" r:id="rId3"/>
-    <sheet name="查询包2参数表" sheetId="4" r:id="rId4"/>
+    <sheet name="常规包1" sheetId="1" r:id="rId1"/>
+    <sheet name="常规包2" sheetId="2" r:id="rId2"/>
+    <sheet name="查询包1" sheetId="3" r:id="rId3"/>
+    <sheet name="帧格式参考(CCSDS)" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1414" uniqueCount="531">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="558">
   <si>
     <t>序号</t>
   </si>
@@ -681,9 +681,6 @@
   </si>
   <si>
     <t>TM1001</t>
-  </si>
-  <si>
-    <t>遥测请求指令计数</t>
   </si>
   <si>
     <t>TM1002</t>
@@ -1683,12 +1680,106 @@
     <t>V</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
+  <si>
+    <t>层级</t>
+  </si>
+  <si>
+    <t>区域</t>
+  </si>
+  <si>
+    <t>字段</t>
+  </si>
+  <si>
+    <t>位宽(bit)</t>
+  </si>
+  <si>
+    <t>说明</t>
+  </si>
+  <si>
+    <t>数据包</t>
+  </si>
+  <si>
+    <t>包主导头</t>
+  </si>
+  <si>
+    <t>标识符</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>固定值</t>
+  </si>
+  <si>
+    <t>版本+类型+副导头+APID</t>
+  </si>
+  <si>
+    <t>0x0520</t>
+  </si>
+  <si>
+    <t>14-bit循环累加</t>
+  </si>
+  <si>
+    <t>数据域长度</t>
+  </si>
+  <si>
+    <t>包数据域</t>
+  </si>
+  <si>
+    <t>不同指令不同值</t>
+  </si>
+  <si>
+    <t>校验和</t>
+  </si>
+  <si>
+    <t>字节3~N求和取反取低16位</t>
+  </si>
+  <si>
+    <t>0x1ACF</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>源包序列号</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>分组标志</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>0b11</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>固定值</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x00~0x3FFF</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>取值范围</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>初始值</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x0001~0x07FF</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>遥测请求指令计数</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1739,6 +1830,29 @@
       <family val="2"/>
       <charset val="134"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1759,7 +1873,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1797,11 +1911,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1822,6 +1951,21 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2126,7 +2270,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S48"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2142,7 +2286,7 @@
     <col min="14" max="14" width="53.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="43.5" customHeight="1">
+    <row r="1" spans="1:14" ht="43.5" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2186,15 +2330,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="14.5" customHeight="1">
+    <row r="2" spans="1:14" ht="14.5" customHeight="1">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>216</v>
+      <c r="C2" s="12" t="s">
+        <v>557</v>
       </c>
       <c r="D2" s="6">
         <v>0</v>
@@ -2224,15 +2368,15 @@
       </c>
       <c r="N2" s="2"/>
     </row>
-    <row r="3" spans="1:19" ht="14.5" customHeight="1">
+    <row r="3" spans="1:14" ht="14.5" customHeight="1">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>217</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>218</v>
       </c>
       <c r="D3" s="6">
         <v>1</v>
@@ -2262,15 +2406,15 @@
       </c>
       <c r="N3" s="2"/>
     </row>
-    <row r="4" spans="1:19" ht="14.5" customHeight="1">
+    <row r="4" spans="1:14" ht="14.5" customHeight="1">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>219</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>220</v>
       </c>
       <c r="D4" s="6">
         <v>2</v>
@@ -2300,15 +2444,15 @@
       </c>
       <c r="N4" s="2"/>
     </row>
-    <row r="5" spans="1:19" ht="14.5" customHeight="1">
+    <row r="5" spans="1:14" ht="14.5" customHeight="1">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>221</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>222</v>
       </c>
       <c r="D5" s="6">
         <v>3</v>
@@ -2338,15 +2482,15 @@
       </c>
       <c r="N5" s="2"/>
     </row>
-    <row r="6" spans="1:19" ht="58" customHeight="1">
+    <row r="6" spans="1:14" ht="58" customHeight="1">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>223</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>224</v>
       </c>
       <c r="D6" s="6">
         <v>5</v>
@@ -2375,22 +2519,18 @@
         <v>15</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
-    </row>
-    <row r="7" spans="1:19" ht="101.5" customHeight="1">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="101.5" customHeight="1">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>226</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>227</v>
       </c>
       <c r="D7" s="6">
         <v>5</v>
@@ -2419,22 +2559,18 @@
         <v>15</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
-    </row>
-    <row r="8" spans="1:19" ht="14.5" customHeight="1">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="14.5" customHeight="1">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>229</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>230</v>
       </c>
       <c r="D8" s="6">
         <v>6</v>
@@ -2463,22 +2599,18 @@
         <v>19</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
-    </row>
-    <row r="9" spans="1:19" ht="14.5" customHeight="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="14.5" customHeight="1">
       <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>232</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>233</v>
       </c>
       <c r="D9" s="6">
         <v>7</v>
@@ -2502,29 +2634,25 @@
         <v>2</v>
       </c>
       <c r="K9" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M9" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="L9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>235</v>
-      </c>
       <c r="N9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="2"/>
-    </row>
-    <row r="10" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="10" spans="1:14" ht="14.5" customHeight="1">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>237</v>
       </c>
       <c r="D10" s="6">
         <v>9</v>
@@ -2548,7 +2676,7 @@
         <v>2</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>18</v>
@@ -2557,20 +2685,16 @@
         <v>58</v>
       </c>
       <c r="N10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
-    </row>
-    <row r="11" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="11" spans="1:14" ht="14.5" customHeight="1">
       <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>239</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>240</v>
       </c>
       <c r="D11" s="6">
         <v>11</v>
@@ -2594,29 +2718,25 @@
         <v>2</v>
       </c>
       <c r="K11" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M11" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="L11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>235</v>
-      </c>
       <c r="N11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
-    </row>
-    <row r="12" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="12" spans="1:14" ht="14.5" customHeight="1">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>241</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>242</v>
       </c>
       <c r="D12" s="6">
         <v>13</v>
@@ -2640,29 +2760,25 @@
         <v>2</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>18</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="N12" s="2"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
-    </row>
-    <row r="13" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="13" spans="1:14" ht="14.5" customHeight="1">
       <c r="A13" s="2">
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>244</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>245</v>
       </c>
       <c r="D13" s="6">
         <v>15</v>
@@ -2686,29 +2802,25 @@
         <v>2</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>18</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="N13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
-    </row>
-    <row r="14" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="14" spans="1:14" ht="14.5" customHeight="1">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>246</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>247</v>
       </c>
       <c r="D14" s="6">
         <v>17</v>
@@ -2732,29 +2844,25 @@
         <v>2</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>18</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="N14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
-    </row>
-    <row r="15" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="15" spans="1:14" ht="14.5" customHeight="1">
       <c r="A15" s="2">
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>248</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>249</v>
       </c>
       <c r="D15" s="6">
         <v>19</v>
@@ -2778,29 +2886,25 @@
         <v>2</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>18</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="N15" s="2"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
-    </row>
-    <row r="16" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="16" spans="1:14" ht="14.5" customHeight="1">
       <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>250</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>251</v>
       </c>
       <c r="D16" s="6">
         <v>21</v>
@@ -2824,29 +2928,25 @@
         <v>2</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>18</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="N16" s="2"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="2"/>
-    </row>
-    <row r="17" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="17" spans="1:14" ht="14.5" customHeight="1">
       <c r="A17" s="2">
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>252</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>253</v>
       </c>
       <c r="D17" s="6">
         <v>23</v>
@@ -2870,7 +2970,7 @@
         <v>2</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>18</v>
@@ -2879,17 +2979,13 @@
         <v>45</v>
       </c>
       <c r="N17" s="2"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="2"/>
-    </row>
-    <row r="18" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="18" spans="1:14" ht="14.5" customHeight="1">
       <c r="A18" s="2">
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>69</v>
@@ -2916,7 +3012,7 @@
         <v>2</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>18</v>
@@ -2925,20 +3021,16 @@
         <v>45</v>
       </c>
       <c r="N18" s="2"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
-      <c r="S18" s="2"/>
-    </row>
-    <row r="19" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="19" spans="1:14" ht="14.5" customHeight="1">
       <c r="A19" s="2">
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>255</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>256</v>
       </c>
       <c r="D19" s="6">
         <v>27</v>
@@ -2962,7 +3054,7 @@
         <v>2</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>18</v>
@@ -2971,17 +3063,13 @@
         <v>45</v>
       </c>
       <c r="N19" s="2"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2"/>
-      <c r="S19" s="2"/>
-    </row>
-    <row r="20" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="20" spans="1:14" ht="14.5" customHeight="1">
       <c r="A20" s="2">
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>69</v>
@@ -3008,7 +3096,7 @@
         <v>2</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>18</v>
@@ -3017,20 +3105,16 @@
         <v>45</v>
       </c>
       <c r="N20" s="2"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-      <c r="R20" s="2"/>
-      <c r="S20" s="2"/>
-    </row>
-    <row r="21" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="21" spans="1:14" ht="14.5" customHeight="1">
       <c r="A21" s="2">
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>258</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>259</v>
       </c>
       <c r="D21" s="6">
         <v>31</v>
@@ -3056,25 +3140,21 @@
         <v>18</v>
       </c>
       <c r="M21" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N21" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="N21" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="2"/>
-      <c r="S21" s="2"/>
-    </row>
-    <row r="22" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="22" spans="1:14" ht="14.5" customHeight="1">
       <c r="A22" s="2">
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>262</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>263</v>
       </c>
       <c r="D22" s="6">
         <v>31</v>
@@ -3100,25 +3180,21 @@
         <v>18</v>
       </c>
       <c r="M22" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N22" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="N22" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="P22" s="2"/>
-      <c r="Q22" s="2"/>
-      <c r="R22" s="2"/>
-      <c r="S22" s="2"/>
-    </row>
-    <row r="23" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="23" spans="1:14" ht="14.5" customHeight="1">
       <c r="A23" s="2">
         <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>264</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>265</v>
       </c>
       <c r="D23" s="6">
         <v>31</v>
@@ -3144,25 +3220,21 @@
         <v>18</v>
       </c>
       <c r="M23" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N23" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="N23" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-      <c r="R23" s="2"/>
-      <c r="S23" s="2"/>
-    </row>
-    <row r="24" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="24" spans="1:14" ht="14.5" customHeight="1">
       <c r="A24" s="2">
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>266</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>267</v>
       </c>
       <c r="D24" s="6">
         <v>31</v>
@@ -3188,25 +3260,21 @@
         <v>18</v>
       </c>
       <c r="M24" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N24" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="N24" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="2"/>
-    </row>
-    <row r="25" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="25" spans="1:14" ht="14.5" customHeight="1">
       <c r="A25" s="2">
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>268</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>269</v>
       </c>
       <c r="D25" s="6">
         <v>32</v>
@@ -3232,21 +3300,21 @@
         <v>18</v>
       </c>
       <c r="M25" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N25" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="N25" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="26" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="26" spans="1:14" ht="14.5" customHeight="1">
       <c r="A26" s="2">
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>270</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>271</v>
       </c>
       <c r="D26" s="6">
         <v>32</v>
@@ -3272,21 +3340,21 @@
         <v>18</v>
       </c>
       <c r="M26" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N26" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="N26" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="27" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="27" spans="1:14" ht="14.5" customHeight="1">
       <c r="A27" s="2">
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>272</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>273</v>
       </c>
       <c r="D27" s="6">
         <v>32</v>
@@ -3312,21 +3380,21 @@
         <v>18</v>
       </c>
       <c r="M27" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N27" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="N27" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="28" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="28" spans="1:14" ht="14.5" customHeight="1">
       <c r="A28" s="2">
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>274</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>275</v>
       </c>
       <c r="D28" s="6">
         <v>32</v>
@@ -3352,21 +3420,21 @@
         <v>18</v>
       </c>
       <c r="M28" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N28" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="N28" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="29" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="29" spans="1:14" ht="14.5" customHeight="1">
       <c r="A29" s="2">
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>276</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>277</v>
       </c>
       <c r="D29" s="6">
         <v>33</v>
@@ -3392,21 +3460,21 @@
         <v>18</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="30" spans="1:19" ht="14.5" customHeight="1">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="14.5" customHeight="1">
       <c r="A30" s="2">
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>278</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>279</v>
       </c>
       <c r="D30" s="6">
         <v>33</v>
@@ -3432,21 +3500,21 @@
         <v>18</v>
       </c>
       <c r="M30" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N30" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="N30" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="31" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="31" spans="1:14" ht="14.5" customHeight="1">
       <c r="A31" s="2">
         <v>30</v>
       </c>
       <c r="B31" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>280</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>281</v>
       </c>
       <c r="D31" s="6">
         <v>33</v>
@@ -3472,21 +3540,21 @@
         <v>18</v>
       </c>
       <c r="M31" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N31" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="N31" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="32" spans="1:19" ht="14.5" customHeight="1">
+    </row>
+    <row r="32" spans="1:14" ht="14.5" customHeight="1">
       <c r="A32" s="2">
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>282</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>283</v>
       </c>
       <c r="D32" s="6">
         <v>33</v>
@@ -3512,10 +3580,10 @@
         <v>18</v>
       </c>
       <c r="M32" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N32" s="2" t="s">
         <v>260</v>
-      </c>
-      <c r="N32" s="2" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="14.5" customHeight="1">
@@ -3523,10 +3591,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>284</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>285</v>
       </c>
       <c r="D33" s="6">
         <v>34</v>
@@ -3555,7 +3623,7 @@
         <v>49</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="14.5" customHeight="1">
@@ -3563,10 +3631,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>287</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>288</v>
       </c>
       <c r="D34" s="6">
         <v>34</v>
@@ -3595,7 +3663,7 @@
         <v>49</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="14.5" customHeight="1">
@@ -3603,10 +3671,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>289</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>290</v>
       </c>
       <c r="D35" s="6">
         <v>34</v>
@@ -3635,7 +3703,7 @@
         <v>49</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="14.5" customHeight="1">
@@ -3643,10 +3711,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>291</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>292</v>
       </c>
       <c r="D36" s="6">
         <v>34</v>
@@ -3675,7 +3743,7 @@
         <v>49</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="14.5" customHeight="1">
@@ -3683,10 +3751,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>293</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>294</v>
       </c>
       <c r="D37" s="6">
         <v>34</v>
@@ -3715,7 +3783,7 @@
         <v>49</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="14.5" customHeight="1">
@@ -3723,10 +3791,10 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>295</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>296</v>
       </c>
       <c r="D38" s="6">
         <v>34</v>
@@ -3755,7 +3823,7 @@
         <v>49</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="14.5" customHeight="1">
@@ -3763,10 +3831,10 @@
         <v>38</v>
       </c>
       <c r="B39" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>297</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>298</v>
       </c>
       <c r="D39" s="6">
         <v>34</v>
@@ -3795,7 +3863,7 @@
         <v>49</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="14.5" customHeight="1">
@@ -3803,10 +3871,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>299</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>300</v>
       </c>
       <c r="D40" s="6">
         <v>34</v>
@@ -3835,7 +3903,7 @@
         <v>49</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="14.5" customHeight="1">
@@ -3843,10 +3911,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>301</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>302</v>
       </c>
       <c r="D41" s="6">
         <v>35</v>
@@ -3875,7 +3943,7 @@
         <v>49</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="14.5" customHeight="1">
@@ -3883,10 +3951,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>303</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>304</v>
       </c>
       <c r="D42" s="6">
         <v>35</v>
@@ -3915,7 +3983,7 @@
         <v>49</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="43" spans="1:14" ht="14.5" customHeight="1">
@@ -3923,10 +3991,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>305</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>306</v>
       </c>
       <c r="D43" s="6">
         <v>35</v>
@@ -3955,7 +4023,7 @@
         <v>49</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="14.5" customHeight="1">
@@ -3963,10 +4031,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>307</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>308</v>
       </c>
       <c r="D44" s="6">
         <v>35</v>
@@ -3995,7 +4063,7 @@
         <v>49</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="14.5" customHeight="1">
@@ -4003,10 +4071,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>309</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>310</v>
       </c>
       <c r="D45" s="6">
         <v>35</v>
@@ -4035,7 +4103,7 @@
         <v>49</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="14.5" customHeight="1">
@@ -4043,10 +4111,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>311</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>312</v>
       </c>
       <c r="D46" s="6">
         <v>35</v>
@@ -4075,7 +4143,7 @@
         <v>49</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="47" spans="1:14" ht="14.5" customHeight="1">
@@ -4083,10 +4151,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>313</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>314</v>
       </c>
       <c r="D47" s="6">
         <v>35</v>
@@ -4115,7 +4183,7 @@
         <v>49</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="48" spans="1:14" ht="14.5" customHeight="1">
@@ -4123,10 +4191,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>315</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>316</v>
       </c>
       <c r="D48" s="6">
         <v>35</v>
@@ -4155,7 +4223,7 @@
         <v>49</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
   </sheetData>
@@ -4470,7 +4538,7 @@
         <v>38</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="D8" s="6">
         <v>11</v>
@@ -4494,7 +4562,7 @@
         <v>2</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>39</v>
@@ -7710,10 +7778,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>318</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>319</v>
       </c>
       <c r="D2" s="6">
         <v>0</v>
@@ -7725,7 +7793,7 @@
         <v>32</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>17</v>
@@ -7744,10 +7812,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>321</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>322</v>
       </c>
       <c r="D3" s="6">
         <v>4</v>
@@ -7759,7 +7827,7 @@
         <v>32</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>17</v>
@@ -7778,10 +7846,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>323</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>324</v>
       </c>
       <c r="D4" s="6">
         <v>8</v>
@@ -7793,7 +7861,7 @@
         <v>32</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>17</v>
@@ -7812,10 +7880,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>325</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>326</v>
       </c>
       <c r="D5" s="6">
         <v>12</v>
@@ -7844,10 +7912,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>327</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>328</v>
       </c>
       <c r="D6" s="6">
         <v>16</v>
@@ -7859,7 +7927,7 @@
         <v>32</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>17</v>
@@ -7878,10 +7946,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>329</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>330</v>
       </c>
       <c r="D7" s="6">
         <v>20</v>
@@ -7893,7 +7961,7 @@
         <v>32</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>17</v>
@@ -7912,10 +7980,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>331</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>332</v>
       </c>
       <c r="D8" s="6">
         <v>24</v>
@@ -7927,7 +7995,7 @@
         <v>32</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>17</v>
@@ -7946,10 +8014,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>333</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>334</v>
       </c>
       <c r="D9" s="6">
         <v>28</v>
@@ -7961,7 +8029,7 @@
         <v>32</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>17</v>
@@ -7980,10 +8048,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>335</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>336</v>
       </c>
       <c r="D10" s="6">
         <v>32</v>
@@ -7995,7 +8063,7 @@
         <v>32</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>17</v>
@@ -8014,10 +8082,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>337</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>338</v>
       </c>
       <c r="D11" s="6">
         <v>36</v>
@@ -8029,7 +8097,7 @@
         <v>32</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>17</v>
@@ -8048,10 +8116,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>339</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>340</v>
       </c>
       <c r="D12" s="6">
         <v>40</v>
@@ -8063,7 +8131,7 @@
         <v>32</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>17</v>
@@ -8082,10 +8150,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>341</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>342</v>
       </c>
       <c r="D13" s="6">
         <v>44</v>
@@ -8097,7 +8165,7 @@
         <v>32</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>17</v>
@@ -8116,10 +8184,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>343</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>344</v>
       </c>
       <c r="D14" s="6">
         <v>48</v>
@@ -8131,7 +8199,7 @@
         <v>32</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>17</v>
@@ -8150,10 +8218,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>345</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>346</v>
       </c>
       <c r="D15" s="6">
         <v>52</v>
@@ -8165,7 +8233,7 @@
         <v>32</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>17</v>
@@ -8184,10 +8252,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>347</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>348</v>
       </c>
       <c r="D16" s="6">
         <v>56</v>
@@ -8199,7 +8267,7 @@
         <v>32</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>17</v>
@@ -8220,10 +8288,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>349</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>350</v>
       </c>
       <c r="D17" s="6">
         <v>60</v>
@@ -8235,7 +8303,7 @@
         <v>32</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>17</v>
@@ -8254,10 +8322,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>351</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>352</v>
       </c>
       <c r="D18" s="6">
         <v>64</v>
@@ -8269,7 +8337,7 @@
         <v>32</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>17</v>
@@ -8286,10 +8354,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>353</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>354</v>
       </c>
       <c r="D19" s="6">
         <v>68</v>
@@ -8320,10 +8388,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>355</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>356</v>
       </c>
       <c r="D20" s="6">
         <v>72</v>
@@ -8354,10 +8422,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>357</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>358</v>
       </c>
       <c r="D21" s="6">
         <v>76</v>
@@ -8369,7 +8437,7 @@
         <v>32</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>17</v>
@@ -8390,10 +8458,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>359</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>360</v>
       </c>
       <c r="D22" s="6">
         <v>80</v>
@@ -8405,7 +8473,7 @@
         <v>32</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>17</v>
@@ -8424,10 +8492,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>361</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>362</v>
       </c>
       <c r="D23" s="6">
         <v>84</v>
@@ -8439,7 +8507,7 @@
         <v>32</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H23" s="6" t="s">
         <v>17</v>
@@ -8458,10 +8526,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>363</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>364</v>
       </c>
       <c r="D24" s="6">
         <v>88</v>
@@ -8473,7 +8541,7 @@
         <v>32</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>17</v>
@@ -8492,10 +8560,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>365</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>366</v>
       </c>
       <c r="D25" s="6">
         <v>92</v>
@@ -8507,7 +8575,7 @@
         <v>32</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>17</v>
@@ -8526,10 +8594,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>367</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>368</v>
       </c>
       <c r="D26" s="6">
         <v>96</v>
@@ -8541,7 +8609,7 @@
         <v>32</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>17</v>
@@ -8560,10 +8628,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>369</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>370</v>
       </c>
       <c r="D27" s="6">
         <v>100</v>
@@ -8575,7 +8643,7 @@
         <v>32</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H27" s="6" t="s">
         <v>17</v>
@@ -8594,10 +8662,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>371</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>372</v>
       </c>
       <c r="D28" s="6">
         <v>104</v>
@@ -8609,7 +8677,7 @@
         <v>32</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>17</v>
@@ -8628,10 +8696,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>373</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>374</v>
       </c>
       <c r="D29" s="6">
         <v>108</v>
@@ -8643,7 +8711,7 @@
         <v>32</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>17</v>
@@ -8662,10 +8730,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>375</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>376</v>
       </c>
       <c r="D30" s="6">
         <v>112</v>
@@ -8677,7 +8745,7 @@
         <v>32</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H30" s="6" t="s">
         <v>17</v>
@@ -8698,10 +8766,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="C31" s="6" t="s">
         <v>377</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>378</v>
       </c>
       <c r="D31" s="6">
         <v>116</v>
@@ -8732,10 +8800,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="C32" s="6" t="s">
         <v>379</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>380</v>
       </c>
       <c r="D32" s="6">
         <v>120</v>
@@ -8747,7 +8815,7 @@
         <v>32</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H32" s="6" t="s">
         <v>17</v>
@@ -8768,10 +8836,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>381</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>382</v>
       </c>
       <c r="D33" s="6">
         <v>124</v>
@@ -8783,7 +8851,7 @@
         <v>32</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>17</v>
@@ -8804,10 +8872,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="C34" s="6" t="s">
         <v>383</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>384</v>
       </c>
       <c r="D34" s="6">
         <v>128</v>
@@ -8819,7 +8887,7 @@
         <v>32</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H34" s="6" t="s">
         <v>17</v>
@@ -8840,10 +8908,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="C35" s="6" t="s">
         <v>385</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>386</v>
       </c>
       <c r="D35" s="6">
         <v>132</v>
@@ -8855,7 +8923,7 @@
         <v>32</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H35" s="6" t="s">
         <v>17</v>
@@ -8876,10 +8944,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>387</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>388</v>
       </c>
       <c r="D36" s="6">
         <v>136</v>
@@ -8891,7 +8959,7 @@
         <v>32</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H36" s="6" t="s">
         <v>17</v>
@@ -8912,10 +8980,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="C37" s="6" t="s">
         <v>389</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>390</v>
       </c>
       <c r="D37" s="6">
         <v>140</v>
@@ -8927,7 +8995,7 @@
         <v>32</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>17</v>
@@ -8948,10 +9016,10 @@
         <v>37</v>
       </c>
       <c r="B38" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>391</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>392</v>
       </c>
       <c r="D38" s="6">
         <v>144</v>
@@ -8963,7 +9031,7 @@
         <v>32</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>17</v>
@@ -8984,10 +9052,10 @@
         <v>38</v>
       </c>
       <c r="B39" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="C39" s="6" t="s">
         <v>393</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>394</v>
       </c>
       <c r="D39" s="6">
         <v>148</v>
@@ -8999,7 +9067,7 @@
         <v>32</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>17</v>
@@ -9020,10 +9088,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>395</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>396</v>
       </c>
       <c r="D40" s="6">
         <v>152</v>
@@ -9035,7 +9103,7 @@
         <v>32</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H40" s="6" t="s">
         <v>17</v>
@@ -9056,10 +9124,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="C41" s="6" t="s">
         <v>397</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>398</v>
       </c>
       <c r="D41" s="6">
         <v>156</v>
@@ -9071,7 +9139,7 @@
         <v>32</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H41" s="6" t="s">
         <v>17</v>
@@ -9090,10 +9158,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="C42" s="6" t="s">
         <v>399</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>400</v>
       </c>
       <c r="D42" s="6">
         <v>160</v>
@@ -9105,7 +9173,7 @@
         <v>32</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H42" s="6" t="s">
         <v>17</v>
@@ -9124,10 +9192,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="C43" s="6" t="s">
         <v>401</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>402</v>
       </c>
       <c r="D43" s="6">
         <v>164</v>
@@ -9139,7 +9207,7 @@
         <v>32</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>17</v>
@@ -9158,10 +9226,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="C44" s="6" t="s">
         <v>403</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>404</v>
       </c>
       <c r="D44" s="6">
         <v>168</v>
@@ -9173,7 +9241,7 @@
         <v>32</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H44" s="6" t="s">
         <v>17</v>
@@ -9192,10 +9260,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="C45" s="6" t="s">
         <v>405</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>406</v>
       </c>
       <c r="D45" s="6">
         <v>172</v>
@@ -9207,7 +9275,7 @@
         <v>32</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H45" s="6" t="s">
         <v>17</v>
@@ -9226,10 +9294,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="6" t="s">
+        <v>406</v>
+      </c>
+      <c r="C46" s="6" t="s">
         <v>407</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>408</v>
       </c>
       <c r="D46" s="6">
         <v>176</v>
@@ -9241,7 +9309,7 @@
         <v>32</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H46" s="6" t="s">
         <v>17</v>
@@ -9260,10 +9328,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="C47" s="6" t="s">
         <v>409</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>410</v>
       </c>
       <c r="D47" s="6">
         <v>180</v>
@@ -9275,7 +9343,7 @@
         <v>32</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H47" s="6" t="s">
         <v>17</v>
@@ -9294,10 +9362,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="C48" s="6" t="s">
         <v>411</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>412</v>
       </c>
       <c r="D48" s="6">
         <v>184</v>
@@ -9309,7 +9377,7 @@
         <v>32</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H48" s="6" t="s">
         <v>17</v>
@@ -9328,10 +9396,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C49" s="6" t="s">
         <v>413</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>414</v>
       </c>
       <c r="D49" s="6">
         <v>188</v>
@@ -9343,7 +9411,7 @@
         <v>32</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H49" s="6" t="s">
         <v>17</v>
@@ -9362,10 +9430,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="C50" s="6" t="s">
         <v>415</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>416</v>
       </c>
       <c r="D50" s="6">
         <v>192</v>
@@ -9377,7 +9445,7 @@
         <v>32</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H50" s="6" t="s">
         <v>17</v>
@@ -9396,10 +9464,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C51" s="6" t="s">
         <v>417</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>418</v>
       </c>
       <c r="D51" s="6">
         <v>196</v>
@@ -9411,7 +9479,7 @@
         <v>32</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H51" s="6" t="s">
         <v>17</v>
@@ -9430,10 +9498,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="C52" s="6" t="s">
         <v>419</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>420</v>
       </c>
       <c r="D52" s="6">
         <v>200</v>
@@ -9445,7 +9513,7 @@
         <v>32</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H52" s="6" t="s">
         <v>17</v>
@@ -9464,10 +9532,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="C53" s="6" t="s">
         <v>421</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>422</v>
       </c>
       <c r="D53" s="6">
         <v>204</v>
@@ -9479,7 +9547,7 @@
         <v>32</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H53" s="6" t="s">
         <v>17</v>
@@ -9498,10 +9566,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="C54" s="6" t="s">
         <v>423</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>424</v>
       </c>
       <c r="D54" s="6">
         <v>208</v>
@@ -9513,7 +9581,7 @@
         <v>32</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H54" s="6" t="s">
         <v>17</v>
@@ -9532,10 +9600,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="6" t="s">
+        <v>424</v>
+      </c>
+      <c r="C55" s="6" t="s">
         <v>425</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>426</v>
       </c>
       <c r="D55" s="6">
         <v>212</v>
@@ -9547,7 +9615,7 @@
         <v>32</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H55" s="6" t="s">
         <v>17</v>
@@ -9566,10 +9634,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="C56" s="6" t="s">
         <v>427</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>428</v>
       </c>
       <c r="D56" s="6">
         <v>216</v>
@@ -9581,7 +9649,7 @@
         <v>32</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H56" s="6" t="s">
         <v>17</v>
@@ -9600,10 +9668,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="6" t="s">
+        <v>428</v>
+      </c>
+      <c r="C57" s="6" t="s">
         <v>429</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>430</v>
       </c>
       <c r="D57" s="6">
         <v>220</v>
@@ -9615,7 +9683,7 @@
         <v>32</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H57" s="6" t="s">
         <v>17</v>
@@ -9634,10 +9702,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="6" t="s">
+        <v>430</v>
+      </c>
+      <c r="C58" s="6" t="s">
         <v>431</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>432</v>
       </c>
       <c r="D58" s="6">
         <v>224</v>
@@ -9649,7 +9717,7 @@
         <v>32</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H58" s="6" t="s">
         <v>17</v>
@@ -9668,10 +9736,10 @@
         <v>58</v>
       </c>
       <c r="B59" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="C59" s="6" t="s">
         <v>433</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>434</v>
       </c>
       <c r="D59" s="6">
         <v>228</v>
@@ -9683,7 +9751,7 @@
         <v>32</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H59" s="6" t="s">
         <v>17</v>
@@ -9702,10 +9770,10 @@
         <v>59</v>
       </c>
       <c r="B60" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="C60" s="6" t="s">
         <v>435</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>436</v>
       </c>
       <c r="D60" s="6">
         <v>232</v>
@@ -9717,7 +9785,7 @@
         <v>32</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H60" s="6" t="s">
         <v>17</v>
@@ -9736,10 +9804,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="C61" s="6" t="s">
         <v>437</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>438</v>
       </c>
       <c r="D61" s="6">
         <v>236</v>
@@ -9751,7 +9819,7 @@
         <v>32</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H61" s="6" t="s">
         <v>17</v>
@@ -9772,10 +9840,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="C62" s="6" t="s">
         <v>439</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>440</v>
       </c>
       <c r="D62" s="6">
         <v>240</v>
@@ -9787,7 +9855,7 @@
         <v>32</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H62" s="6" t="s">
         <v>17</v>
@@ -9808,10 +9876,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="6" t="s">
+        <v>440</v>
+      </c>
+      <c r="C63" s="6" t="s">
         <v>441</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>442</v>
       </c>
       <c r="D63" s="6">
         <v>244</v>
@@ -9823,7 +9891,7 @@
         <v>32</v>
       </c>
       <c r="G63" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H63" s="6" t="s">
         <v>17</v>
@@ -9844,10 +9912,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="C64" s="6" t="s">
         <v>443</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>444</v>
       </c>
       <c r="D64" s="6">
         <v>248</v>
@@ -9859,7 +9927,7 @@
         <v>32</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H64" s="6" t="s">
         <v>17</v>
@@ -9880,10 +9948,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="C65" s="6" t="s">
         <v>445</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>446</v>
       </c>
       <c r="D65" s="6">
         <v>252</v>
@@ -9895,7 +9963,7 @@
         <v>32</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H65" s="6" t="s">
         <v>17</v>
@@ -9914,10 +9982,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C66" s="6" t="s">
         <v>447</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>448</v>
       </c>
       <c r="D66" s="6">
         <v>256</v>
@@ -9929,7 +9997,7 @@
         <v>32</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H66" s="6" t="s">
         <v>17</v>
@@ -9950,10 +10018,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="C67" s="6" t="s">
         <v>449</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>450</v>
       </c>
       <c r="D67" s="6">
         <v>260</v>
@@ -9965,7 +10033,7 @@
         <v>32</v>
       </c>
       <c r="G67" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H67" s="6" t="s">
         <v>17</v>
@@ -9984,10 +10052,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="C68" s="6" t="s">
         <v>451</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>452</v>
       </c>
       <c r="D68" s="6">
         <v>264</v>
@@ -9999,7 +10067,7 @@
         <v>32</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H68" s="6" t="s">
         <v>17</v>
@@ -10020,10 +10088,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="6" t="s">
+        <v>452</v>
+      </c>
+      <c r="C69" s="6" t="s">
         <v>453</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>454</v>
       </c>
       <c r="D69" s="6">
         <v>268</v>
@@ -10035,7 +10103,7 @@
         <v>32</v>
       </c>
       <c r="G69" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H69" s="6" t="s">
         <v>17</v>
@@ -10054,10 +10122,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C70" s="6" t="s">
         <v>455</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>456</v>
       </c>
       <c r="D70" s="6">
         <v>272</v>
@@ -10069,7 +10137,7 @@
         <v>32</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>17</v>
@@ -10088,10 +10156,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="C71" s="6" t="s">
         <v>457</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>458</v>
       </c>
       <c r="D71" s="6">
         <v>276</v>
@@ -10103,7 +10171,7 @@
         <v>32</v>
       </c>
       <c r="G71" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H71" s="6" t="s">
         <v>17</v>
@@ -10122,10 +10190,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="C72" s="6" t="s">
         <v>459</v>
-      </c>
-      <c r="C72" s="6" t="s">
-        <v>460</v>
       </c>
       <c r="D72" s="6">
         <v>280</v>
@@ -10137,7 +10205,7 @@
         <v>32</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H72" s="6" t="s">
         <v>17</v>
@@ -10158,10 +10226,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="6" t="s">
+        <v>460</v>
+      </c>
+      <c r="C73" s="6" t="s">
         <v>461</v>
-      </c>
-      <c r="C73" s="6" t="s">
-        <v>462</v>
       </c>
       <c r="D73" s="6">
         <v>284</v>
@@ -10173,7 +10241,7 @@
         <v>32</v>
       </c>
       <c r="G73" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H73" s="6" t="s">
         <v>17</v>
@@ -10183,7 +10251,7 @@
         <v>6</v>
       </c>
       <c r="K73" s="6" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L73" s="6"/>
       <c r="M73" s="6"/>
@@ -10194,10 +10262,10 @@
         <v>73</v>
       </c>
       <c r="B74" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="C74" s="6" t="s">
         <v>464</v>
-      </c>
-      <c r="C74" s="6" t="s">
-        <v>465</v>
       </c>
       <c r="D74" s="6">
         <v>288</v>
@@ -10209,7 +10277,7 @@
         <v>32</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H74" s="6" t="s">
         <v>17</v>
@@ -10219,7 +10287,7 @@
         <v>6</v>
       </c>
       <c r="K74" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L74" s="6"/>
       <c r="M74" s="6"/>
@@ -10230,10 +10298,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="C75" s="6" t="s">
         <v>466</v>
-      </c>
-      <c r="C75" s="6" t="s">
-        <v>467</v>
       </c>
       <c r="D75" s="6">
         <v>292</v>
@@ -10245,7 +10313,7 @@
         <v>32</v>
       </c>
       <c r="G75" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H75" s="6" t="s">
         <v>17</v>
@@ -10266,10 +10334,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="C76" s="6" t="s">
         <v>468</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>469</v>
       </c>
       <c r="D76" s="6">
         <v>296</v>
@@ -10281,7 +10349,7 @@
         <v>32</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H76" s="6" t="s">
         <v>17</v>
@@ -10291,7 +10359,7 @@
         <v>6</v>
       </c>
       <c r="K76" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L76" s="6"/>
       <c r="M76" s="6">
@@ -10304,10 +10372,10 @@
         <v>76</v>
       </c>
       <c r="B77" s="6" t="s">
+        <v>469</v>
+      </c>
+      <c r="C77" s="6" t="s">
         <v>470</v>
-      </c>
-      <c r="C77" s="6" t="s">
-        <v>471</v>
       </c>
       <c r="D77" s="6">
         <v>300</v>
@@ -10319,7 +10387,7 @@
         <v>32</v>
       </c>
       <c r="G77" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H77" s="6" t="s">
         <v>17</v>
@@ -10329,7 +10397,7 @@
         <v>6</v>
       </c>
       <c r="K77" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L77" s="6"/>
       <c r="M77" s="6">
@@ -10342,10 +10410,10 @@
         <v>77</v>
       </c>
       <c r="B78" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="C78" s="6" t="s">
         <v>472</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>473</v>
       </c>
       <c r="D78" s="6">
         <v>304</v>
@@ -10357,7 +10425,7 @@
         <v>32</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H78" s="6" t="s">
         <v>17</v>
@@ -10367,7 +10435,7 @@
         <v>6</v>
       </c>
       <c r="K78" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L78" s="6"/>
       <c r="M78" s="6">
@@ -10380,10 +10448,10 @@
         <v>78</v>
       </c>
       <c r="B79" s="6" t="s">
+        <v>473</v>
+      </c>
+      <c r="C79" s="6" t="s">
         <v>474</v>
-      </c>
-      <c r="C79" s="6" t="s">
-        <v>475</v>
       </c>
       <c r="D79" s="6">
         <v>308</v>
@@ -10395,7 +10463,7 @@
         <v>32</v>
       </c>
       <c r="G79" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H79" s="6" t="s">
         <v>17</v>
@@ -10405,7 +10473,7 @@
         <v>6</v>
       </c>
       <c r="K79" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L79" s="6"/>
       <c r="M79" s="6">
@@ -10418,10 +10486,10 @@
         <v>79</v>
       </c>
       <c r="B80" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="C80" s="6" t="s">
         <v>476</v>
-      </c>
-      <c r="C80" s="6" t="s">
-        <v>477</v>
       </c>
       <c r="D80" s="6">
         <v>312</v>
@@ -10433,7 +10501,7 @@
         <v>32</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H80" s="6" t="s">
         <v>17</v>
@@ -10443,7 +10511,7 @@
         <v>6</v>
       </c>
       <c r="K80" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L80" s="6"/>
       <c r="M80" s="6">
@@ -10456,10 +10524,10 @@
         <v>80</v>
       </c>
       <c r="B81" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="C81" s="6" t="s">
         <v>478</v>
-      </c>
-      <c r="C81" s="6" t="s">
-        <v>479</v>
       </c>
       <c r="D81" s="6">
         <v>316</v>
@@ -10471,7 +10539,7 @@
         <v>32</v>
       </c>
       <c r="G81" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H81" s="6" t="s">
         <v>17</v>
@@ -10481,7 +10549,7 @@
         <v>6</v>
       </c>
       <c r="K81" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L81" s="6"/>
       <c r="M81" s="6">
@@ -10494,10 +10562,10 @@
         <v>81</v>
       </c>
       <c r="B82" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="C82" s="6" t="s">
         <v>480</v>
-      </c>
-      <c r="C82" s="6" t="s">
-        <v>481</v>
       </c>
       <c r="D82" s="6">
         <v>320</v>
@@ -10509,7 +10577,7 @@
         <v>32</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H82" s="6" t="s">
         <v>17</v>
@@ -10519,7 +10587,7 @@
         <v>6</v>
       </c>
       <c r="K82" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L82" s="6"/>
       <c r="M82" s="6">
@@ -10532,10 +10600,10 @@
         <v>82</v>
       </c>
       <c r="B83" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="C83" s="6" t="s">
         <v>482</v>
-      </c>
-      <c r="C83" s="6" t="s">
-        <v>483</v>
       </c>
       <c r="D83" s="6">
         <v>324</v>
@@ -10547,7 +10615,7 @@
         <v>32</v>
       </c>
       <c r="G83" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H83" s="6" t="s">
         <v>17</v>
@@ -10557,7 +10625,7 @@
         <v>6</v>
       </c>
       <c r="K83" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L83" s="6"/>
       <c r="M83" s="6">
@@ -10570,10 +10638,10 @@
         <v>83</v>
       </c>
       <c r="B84" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="C84" s="6" t="s">
         <v>484</v>
-      </c>
-      <c r="C84" s="6" t="s">
-        <v>485</v>
       </c>
       <c r="D84" s="6">
         <v>328</v>
@@ -10585,7 +10653,7 @@
         <v>32</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H84" s="6" t="s">
         <v>17</v>
@@ -10595,7 +10663,7 @@
         <v>6</v>
       </c>
       <c r="K84" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L84" s="6"/>
       <c r="M84" s="6"/>
@@ -10606,10 +10674,10 @@
         <v>84</v>
       </c>
       <c r="B85" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="C85" s="6" t="s">
         <v>486</v>
-      </c>
-      <c r="C85" s="6" t="s">
-        <v>487</v>
       </c>
       <c r="D85" s="6">
         <v>332</v>
@@ -10621,7 +10689,7 @@
         <v>32</v>
       </c>
       <c r="G85" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H85" s="6" t="s">
         <v>17</v>
@@ -10631,7 +10699,7 @@
         <v>6</v>
       </c>
       <c r="K85" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L85" s="6"/>
       <c r="M85" s="6"/>
@@ -10642,10 +10710,10 @@
         <v>85</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D86" s="6">
         <v>336</v>
@@ -10657,7 +10725,7 @@
         <v>32</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H86" s="6" t="s">
         <v>17</v>
@@ -10667,7 +10735,7 @@
         <v>6</v>
       </c>
       <c r="K86" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L86" s="6"/>
       <c r="M86" s="6">
@@ -10680,10 +10748,10 @@
         <v>86</v>
       </c>
       <c r="B87" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="C87" s="6" t="s">
         <v>489</v>
-      </c>
-      <c r="C87" s="6" t="s">
-        <v>490</v>
       </c>
       <c r="D87" s="6">
         <v>340</v>
@@ -10695,7 +10763,7 @@
         <v>32</v>
       </c>
       <c r="G87" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H87" s="6" t="s">
         <v>17</v>
@@ -10716,10 +10784,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="C88" s="6" t="s">
         <v>491</v>
-      </c>
-      <c r="C88" s="6" t="s">
-        <v>492</v>
       </c>
       <c r="D88" s="6">
         <v>344</v>
@@ -10731,7 +10799,7 @@
         <v>32</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H88" s="6" t="s">
         <v>17</v>
@@ -10754,10 +10822,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="C89" s="6" t="s">
         <v>493</v>
-      </c>
-      <c r="C89" s="6" t="s">
-        <v>494</v>
       </c>
       <c r="D89" s="6">
         <v>348</v>
@@ -10769,7 +10837,7 @@
         <v>32</v>
       </c>
       <c r="G89" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H89" s="6" t="s">
         <v>17</v>
@@ -10792,10 +10860,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="C90" s="6" t="s">
         <v>495</v>
-      </c>
-      <c r="C90" s="6" t="s">
-        <v>496</v>
       </c>
       <c r="D90" s="6">
         <v>352</v>
@@ -10807,7 +10875,7 @@
         <v>32</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H90" s="6" t="s">
         <v>17</v>
@@ -10817,7 +10885,7 @@
         <v>6</v>
       </c>
       <c r="K90" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L90" s="6"/>
       <c r="M90" s="6">
@@ -10830,10 +10898,10 @@
         <v>90</v>
       </c>
       <c r="B91" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="C91" s="6" t="s">
         <v>497</v>
-      </c>
-      <c r="C91" s="6" t="s">
-        <v>498</v>
       </c>
       <c r="D91" s="6">
         <v>356</v>
@@ -10845,7 +10913,7 @@
         <v>32</v>
       </c>
       <c r="G91" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H91" s="6" t="s">
         <v>17</v>
@@ -10866,10 +10934,10 @@
         <v>91</v>
       </c>
       <c r="B92" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C92" s="6" t="s">
         <v>499</v>
-      </c>
-      <c r="C92" s="6" t="s">
-        <v>500</v>
       </c>
       <c r="D92" s="6">
         <v>360</v>
@@ -10881,7 +10949,7 @@
         <v>32</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H92" s="6" t="s">
         <v>17</v>
@@ -10904,10 +10972,10 @@
         <v>92</v>
       </c>
       <c r="B93" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="C93" s="6" t="s">
         <v>501</v>
-      </c>
-      <c r="C93" s="6" t="s">
-        <v>502</v>
       </c>
       <c r="D93" s="6">
         <v>364</v>
@@ -10919,7 +10987,7 @@
         <v>32</v>
       </c>
       <c r="G93" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H93" s="6" t="s">
         <v>17</v>
@@ -10942,10 +11010,10 @@
         <v>93</v>
       </c>
       <c r="B94" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="C94" s="6" t="s">
         <v>503</v>
-      </c>
-      <c r="C94" s="6" t="s">
-        <v>504</v>
       </c>
       <c r="D94" s="6">
         <v>368</v>
@@ -10969,7 +11037,7 @@
         <v>2</v>
       </c>
       <c r="K94" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L94" s="6"/>
       <c r="M94" s="6"/>
@@ -10980,10 +11048,10 @@
         <v>94</v>
       </c>
       <c r="B95" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="C95" s="6" t="s">
         <v>505</v>
-      </c>
-      <c r="C95" s="6" t="s">
-        <v>506</v>
       </c>
       <c r="D95" s="6">
         <v>370</v>
@@ -11007,7 +11075,7 @@
         <v>2</v>
       </c>
       <c r="K95" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L95" s="6"/>
       <c r="M95" s="6">
@@ -11020,10 +11088,10 @@
         <v>95</v>
       </c>
       <c r="B96" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="C96" s="6" t="s">
         <v>507</v>
-      </c>
-      <c r="C96" s="6" t="s">
-        <v>508</v>
       </c>
       <c r="D96" s="6">
         <v>372</v>
@@ -11060,10 +11128,10 @@
         <v>96</v>
       </c>
       <c r="B97" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="C97" s="6" t="s">
         <v>509</v>
-      </c>
-      <c r="C97" s="6" t="s">
-        <v>510</v>
       </c>
       <c r="D97" s="6">
         <v>374</v>
@@ -11096,10 +11164,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="6" t="s">
+        <v>510</v>
+      </c>
+      <c r="C98" s="6" t="s">
         <v>511</v>
-      </c>
-      <c r="C98" s="6" t="s">
-        <v>512</v>
       </c>
       <c r="D98" s="6">
         <v>376</v>
@@ -11130,10 +11198,10 @@
         <v>98</v>
       </c>
       <c r="B99" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="C99" s="6" t="s">
         <v>513</v>
-      </c>
-      <c r="C99" s="6" t="s">
-        <v>514</v>
       </c>
       <c r="D99" s="6">
         <v>378</v>
@@ -11157,7 +11225,7 @@
         <v>2</v>
       </c>
       <c r="K99" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L99" s="6"/>
       <c r="M99" s="6">
@@ -11170,10 +11238,10 @@
         <v>99</v>
       </c>
       <c r="B100" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="C100" s="6" t="s">
         <v>515</v>
-      </c>
-      <c r="C100" s="6" t="s">
-        <v>516</v>
       </c>
       <c r="D100" s="6">
         <v>380</v>
@@ -11208,10 +11276,10 @@
         <v>100</v>
       </c>
       <c r="B101" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="C101" s="6" t="s">
         <v>517</v>
-      </c>
-      <c r="C101" s="6" t="s">
-        <v>518</v>
       </c>
       <c r="D101" s="6">
         <v>382</v>
@@ -11235,7 +11303,7 @@
         <v>2</v>
       </c>
       <c r="K101" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L101" s="6"/>
       <c r="M101" s="6"/>
@@ -11246,10 +11314,10 @@
         <v>101</v>
       </c>
       <c r="B102" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="C102" s="6" t="s">
         <v>519</v>
-      </c>
-      <c r="C102" s="6" t="s">
-        <v>520</v>
       </c>
       <c r="D102" s="6">
         <v>384</v>
@@ -11280,10 +11348,10 @@
         <v>102</v>
       </c>
       <c r="B103" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="C103" s="6" t="s">
         <v>521</v>
-      </c>
-      <c r="C103" s="6" t="s">
-        <v>522</v>
       </c>
       <c r="D103" s="6">
         <v>386</v>
@@ -11307,7 +11375,7 @@
         <v>2</v>
       </c>
       <c r="K103" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L103" s="6"/>
       <c r="M103" s="6"/>
@@ -11318,10 +11386,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="C104" s="6" t="s">
         <v>523</v>
-      </c>
-      <c r="C104" s="6" t="s">
-        <v>524</v>
       </c>
       <c r="D104" s="6">
         <v>388</v>
@@ -11354,10 +11422,10 @@
         <v>104</v>
       </c>
       <c r="B105" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="C105" s="6" t="s">
         <v>525</v>
-      </c>
-      <c r="C105" s="6" t="s">
-        <v>526</v>
       </c>
       <c r="D105" s="6">
         <v>390</v>
@@ -11388,7 +11456,7 @@
         <v>105</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C106" s="6" t="s">
         <v>69</v>
@@ -11423,52 +11491,158 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEFBA2A6-6BDF-41AF-BB34-FDE1795B9803}">
-  <dimension ref="A1:N1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24C3F8CB-24AA-47EC-AECD-BD359B2FEDB4}">
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="3" max="3" width="27.26953125" customWidth="1"/>
+    <col min="5" max="6" width="14.7265625" customWidth="1"/>
+    <col min="7" max="7" width="25.6328125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="58">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:7" ht="16.5">
+      <c r="A1" s="8" t="s">
+        <v>530</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>533</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>555</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>554</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="9" t="s">
+        <v>535</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>536</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>548</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9" t="s">
+        <v>540</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>541</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>539</v>
+      </c>
+      <c r="G3" s="9"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9" t="s">
+        <v>550</v>
+      </c>
+      <c r="D4" s="9">
+        <v>2</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>551</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>539</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9" t="s">
+        <v>549</v>
+      </c>
+      <c r="D5" s="9">
+        <v>14</v>
+      </c>
+      <c r="E5">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="5" t="s">
+      <c r="F5" s="9" t="s">
+        <v>553</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9" t="s">
+        <v>543</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9" t="s">
+        <v>556</v>
+      </c>
+      <c r="G6" s="9"/>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="9" t="s">
+        <v>535</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>544</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>557</v>
+      </c>
+      <c r="D7" s="9">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>13</v>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9" t="s">
+        <v>546</v>
+      </c>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9" t="s">
+        <v>547</v>
       </c>
     </row>
   </sheetData>

</xml_diff>